<commit_message>
CRM: log Steve's 10/16 post-visit email to Accial (unanswered); next action = deliver items 14/15 with timing ask
</commit_message>
<xml_diff>
--- a/Analyses (internal)/i2c Network Transactions by Month_20260911.xlsx
+++ b/Analyses (internal)/i2c Network Transactions by Month_20260911.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stevenabraham/apps/zed/debt_dd/Analyses (internal)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B636CE41-8188-9944-B94D-40C496EE68AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05AFD5E3-0A11-8841-AF92-460F4AB0D6B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="36000" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="58100" yWindow="3700" windowWidth="36000" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Network Transactions" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" calcMode="autoNoTable" iterate="1"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>i2c invoices — PIN POS &amp; ATM + Signature transactions per month</t>
   </si>
@@ -108,6 +109,9 @@
   </si>
   <si>
     <t>Net Interchange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can </t>
   </si>
 </sst>
 </file>
@@ -219,14 +223,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="5" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="5" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="5" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="5" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -547,16 +551,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="3" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+    </row>
+    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -625,14 +629,14 @@
         <f>H4-G4</f>
         <v>13574.101863799284</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="7">
         <v>1035457.6372759859</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="9">
         <f>H4/J4</f>
         <v>1.5202091613530415E-2</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="9">
         <f>I4/J4</f>
         <v>1.3109277845020431E-2</v>
       </c>
@@ -668,14 +672,14 @@
         <f t="shared" ref="I5:I14" si="2">H5-G5</f>
         <v>13882.415197132617</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="7">
         <v>1165190.9078853049</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="9">
         <f t="shared" ref="K5:K15" si="3">H5/J5</f>
         <v>1.3951580884402846E-2</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <f t="shared" ref="L5:L15" si="4">I5/J5</f>
         <v>1.1914283833820583E-2</v>
       </c>
@@ -711,14 +715,14 @@
         <f t="shared" si="2"/>
         <v>13179.49594982079</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="7">
         <v>1232228.4835125445</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="9">
         <f t="shared" si="3"/>
         <v>1.296157016618598E-2</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="9">
         <f t="shared" si="4"/>
         <v>1.0695659227298341E-2</v>
       </c>
@@ -754,14 +758,14 @@
         <f t="shared" si="2"/>
         <v>15874.983584229391</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="8">
         <v>1298551.8765232973</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="9">
         <f t="shared" si="3"/>
         <v>1.4563764394891385E-2</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="9">
         <f t="shared" si="4"/>
         <v>1.2225143924732973E-2</v>
       </c>
@@ -797,14 +801,14 @@
         <f t="shared" si="2"/>
         <v>11716.816738351255</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="7">
         <v>1116300.5179211472</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="9">
         <f t="shared" si="3"/>
         <v>1.2850739122710477E-2</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="9">
         <f t="shared" si="4"/>
         <v>1.0496113322755712E-2</v>
       </c>
@@ -840,14 +844,14 @@
         <f t="shared" si="2"/>
         <v>12540.265053763444</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="7">
         <v>1191698.214336918</v>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="9">
         <f t="shared" si="3"/>
         <v>1.3002633441374463E-2</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="9">
         <f t="shared" si="4"/>
         <v>1.0523020763894548E-2</v>
       </c>
@@ -883,14 +887,14 @@
         <f t="shared" si="2"/>
         <v>20232.583476702508</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="7">
         <v>1868752.4822580642</v>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="9">
         <f t="shared" si="3"/>
         <v>1.3086577119700828E-2</v>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="9">
         <f t="shared" si="4"/>
         <v>1.0826786141444975E-2</v>
       </c>
@@ -926,14 +930,14 @@
         <f t="shared" si="2"/>
         <v>22251.586487455199</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="7">
         <v>2063789.8666666662</v>
       </c>
-      <c r="K11" s="11">
+      <c r="K11" s="9">
         <f t="shared" si="3"/>
         <v>1.3212399638097136E-2</v>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="9">
         <f t="shared" si="4"/>
         <v>1.0781905099376656E-2</v>
       </c>
@@ -969,14 +973,14 @@
         <f t="shared" si="2"/>
         <v>22045.296021505375</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="7">
         <v>2325289.8025089661</v>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="9">
         <f t="shared" si="3"/>
         <v>1.1912100587040085E-2</v>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="9">
         <f t="shared" si="4"/>
         <v>9.4806660218088538E-3</v>
       </c>
@@ -1012,14 +1016,14 @@
         <f t="shared" si="2"/>
         <v>28984.498172043008</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="7">
         <v>2524444.7741935491</v>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="9">
         <f t="shared" si="3"/>
         <v>1.3936802473043745E-2</v>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="9">
         <f t="shared" si="4"/>
         <v>1.1481533867700592E-2</v>
       </c>
@@ -1029,34 +1033,34 @@
         <v>17</v>
       </c>
       <c r="B14" s="5">
-        <f>SUM(B4:B13)</f>
+        <f t="shared" ref="B14:H14" si="5">SUM(B4:B13)</f>
         <v>120</v>
       </c>
       <c r="C14" s="5">
-        <f>SUM(C4:C13)</f>
+        <f t="shared" si="5"/>
         <v>1336605</v>
       </c>
       <c r="D14" s="5">
-        <f>SUM(D4:D13)</f>
+        <f t="shared" si="5"/>
         <v>1336725</v>
       </c>
       <c r="E14" s="6">
-        <f>SUM(E4:E13)</f>
+        <f t="shared" si="5"/>
         <v>3.3200000000000003</v>
       </c>
       <c r="F14" s="6">
-        <f>SUM(F4:F13)</f>
+        <f t="shared" si="5"/>
         <v>37040.899999999994</v>
       </c>
       <c r="G14" s="6">
-        <f>SUM(G4:G13)</f>
+        <f t="shared" si="5"/>
         <v>37044.22</v>
       </c>
       <c r="H14" s="6">
-        <f>SUM(H4:H13)</f>
+        <f t="shared" si="5"/>
         <v>211326.26254480288</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="10">
         <f t="shared" si="2"/>
         <v>174282.04254480288</v>
       </c>
@@ -1064,11 +1068,11 @@
         <f>SUM(J4:J13)</f>
         <v>15821704.563082444</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="9">
         <f t="shared" si="3"/>
         <v>1.3356731678450169E-2</v>
       </c>
-      <c r="L14" s="11">
+      <c r="L14" s="9">
         <f t="shared" si="4"/>
         <v>1.1015377126397852E-2</v>
       </c>
@@ -1078,36 +1082,41 @@
         <v>23</v>
       </c>
       <c r="E15" s="3">
-        <f>SUM(E8:E13)</f>
+        <f t="shared" ref="E15:J15" si="6">SUM(E8:E13)</f>
         <v>2.2999999999999998</v>
       </c>
       <c r="F15" s="3">
-        <f>SUM(F8:F13)</f>
+        <f t="shared" si="6"/>
         <v>26672.12</v>
       </c>
       <c r="G15" s="3">
-        <f>SUM(G8:G13)</f>
+        <f t="shared" si="6"/>
         <v>26674.42</v>
       </c>
       <c r="H15" s="3">
-        <f>SUM(H8:H13)</f>
+        <f t="shared" si="6"/>
         <v>144445.46594982079</v>
       </c>
       <c r="I15" s="3">
-        <f>SUM(I8:I13)</f>
+        <f t="shared" si="6"/>
         <v>117771.04594982078</v>
       </c>
       <c r="J15" s="3">
-        <f>SUM(J8:J13)</f>
+        <f t="shared" si="6"/>
         <v>11090275.657885311</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="9">
         <f t="shared" si="3"/>
         <v>1.3024515386785578E-2</v>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="9">
         <f t="shared" si="4"/>
         <v>1.0619307362850286E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>